<commit_message>
Add top gaming studios to centralized company catalog
</commit_message>
<xml_diff>
--- a/Careers Sites.xlsx
+++ b/Careers Sites.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K191"/>
+  <dimension ref="A1:K210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10345,6 +10345,443 @@
           <t>Active (200)</t>
         </is>
       </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Rockstar Games</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>https://www.rockstargames.com/careers</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Krafton India</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>https://krafton.in/careers/</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Scopely</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>https://scopely.com/careers/</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Zynga</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>https://www.zynga.com/careers/</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Ubisoft India</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>https://www.ubisoft.com/en-us/company/careers</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Pune / Mumbai)</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Keywords Studios / Lakshya Digital</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>https://www.keywordsstudios.com/en/careers/</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Game QA &amp; Art (Bangalore/Gurgaon)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Gameloft</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>https://www.gameloft.com/corporate/en/jobs/</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Gaming Studio</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Unity Technologies</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>https://careers.unity.com/</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Game Engine Platform (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Sony PlayStation</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>https://playstation.careers/</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Console &amp; Gaming Platform</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Epic Games</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>https://www.epicgames.com/site/en-US/careers</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Unreal Engine &amp; Gaming</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Riot Games</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>https://www.riotgames.com/en/work-with-us/offices/india</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Gaming Studio (India)</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>PlaySimple Games</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>https://careers.playsimple.in/</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Mobile Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Moonfrog Labs (Stillfront)</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>https://moonfroglabs.com/careers/</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Mobile Gaming Studio (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Games24x7</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>https://www.games24x7.com/careers/</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Online Gaming (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Mobile Premier League (MPL)</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>https://www.mpl.live/careers</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Esports &amp; Gaming (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Dream11 (Dream Sports)</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>https://careers.dreamsports.group/</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Sports Tech &amp; Gaming</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>PTW (Pole To Win)</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>https://www.ptw.com/careers</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Game QA &amp; Localization (Bangalore/Hyderabad)</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Electronic Arts (EA India)</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>https://www.ea.com/careers</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Gaming Studio (Hyderabad)</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Junglee Games</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>https://www.jungleegames.com/careers</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Online Gaming (Bangalore)</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>